<commit_message>
Relatório da semana 2026-10-18
</commit_message>
<xml_diff>
--- a/reports/2026-10-18/relatorio.xlsx
+++ b/reports/2026-10-18/relatorio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico Brasil" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados (semana)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paridade etanol" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Histórico Brasil" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estados (semana)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Paridade etanol" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1791,12 +1791,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -2607,17 +2607,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>7.43</v>
+        <v>7.44</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>6.99</v>
+        <v>7.18</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>8.26</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="G28" t="n">
         <v>15</v>
@@ -2636,20 +2636,20 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>6.64</v>
+        <v>6.93</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>6.28</v>
+        <v>6.38</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>7.67</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="G29" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30">
@@ -2665,20 +2665,20 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>6.35</v>
+        <v>6.5</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>6.24</v>
+        <v>6.45</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>6.85</v>
       </c>
       <c r="G30" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -2694,11 +2694,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>7.03</v>
+        <v>7.09</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>6.88</v>
@@ -2707,7 +2707,7 @@
         <v>8.99</v>
       </c>
       <c r="G31" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32">
@@ -2723,20 +2723,20 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>6.7</v>
+        <v>6.86</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>6.13</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>9.92</v>
+        <v>7.78</v>
       </c>
       <c r="G32" t="n">
-        <v>224</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33">
@@ -2752,20 +2752,20 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>6.94</v>
+        <v>7.09</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>5.84</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>7.38</v>
+        <v>7.99</v>
       </c>
       <c r="G33" t="n">
-        <v>139</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34">
@@ -2781,20 +2781,20 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>6.39</v>
+        <v>6.53</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>6.15</v>
+        <v>6.28</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>6.69</v>
+        <v>7.15</v>
       </c>
       <c r="G34" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35">
@@ -2810,20 +2810,20 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>6.39</v>
+        <v>6.62</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>6.03</v>
+        <v>6.09</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>7.23</v>
+        <v>7.53</v>
       </c>
       <c r="G35" t="n">
-        <v>92</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36">
@@ -2839,20 +2839,20 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>6.42</v>
+        <v>6.65</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>5.69</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>6.9</v>
+        <v>7.49</v>
       </c>
       <c r="G36" t="n">
-        <v>189</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37">
@@ -2868,20 +2868,20 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>6.52</v>
+        <v>6.65</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>6.04</v>
+        <v>6.23</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>7.54</v>
       </c>
       <c r="G37" t="n">
-        <v>115</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38">
@@ -2897,20 +2897,20 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>6.75</v>
+        <v>6.95</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>5.83</v>
+        <v>6.45</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>7.19</v>
+        <v>7.49</v>
       </c>
       <c r="G38" t="n">
-        <v>69</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39">
@@ -2926,20 +2926,20 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>6.4</v>
+        <v>6.59</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>6.07</v>
+        <v>6.11</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>7.29</v>
+        <v>7.49</v>
       </c>
       <c r="G39" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40">
@@ -2955,20 +2955,20 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>6.32</v>
+        <v>6.57</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>5.64</v>
+        <v>5.72</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>7.19</v>
+        <v>7.39</v>
       </c>
       <c r="G40" t="n">
-        <v>484</v>
+        <v>314</v>
       </c>
     </row>
     <row r="41">
@@ -2984,20 +2984,20 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>6.58</v>
+        <v>6.8</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>5.81</v>
+        <v>5.94</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>7.7</v>
+        <v>7.89</v>
       </c>
       <c r="G41" t="n">
-        <v>117</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42">
@@ -3013,20 +3013,20 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>6.31</v>
+        <v>6.52</v>
       </c>
       <c r="E42" s="3" t="n">
         <v>6.19</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>6.87</v>
+        <v>6.84</v>
       </c>
       <c r="G42" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
     </row>
     <row r="43">
@@ -3042,20 +3042,20 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>6.57</v>
+        <v>6.77</v>
       </c>
       <c r="E43" s="3" t="n">
         <v>5.59</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>7.38</v>
+        <v>7.39</v>
       </c>
       <c r="G43" t="n">
-        <v>291</v>
+        <v>231</v>
       </c>
     </row>
     <row r="44">
@@ -3071,20 +3071,20 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>6.88</v>
+        <v>7.05</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>6.13</v>
+        <v>6.14</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>7.99</v>
+        <v>7.74</v>
       </c>
       <c r="G44" t="n">
-        <v>192</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45">
@@ -3100,20 +3100,20 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>6.71</v>
+        <v>6.91</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>6.19</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>6.99</v>
+        <v>7.39</v>
       </c>
       <c r="G45" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46">
@@ -3129,20 +3129,20 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>6.59</v>
+        <v>6.8</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>6.08</v>
+        <v>6.15</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>7.39</v>
+        <v>7.99</v>
       </c>
       <c r="G46" t="n">
-        <v>322</v>
+        <v>288</v>
       </c>
     </row>
     <row r="47">
@@ -3158,20 +3158,20 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>6.76</v>
+        <v>6.84</v>
       </c>
       <c r="E47" s="3" t="n">
         <v>6.22</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>7.59</v>
+        <v>7.29</v>
       </c>
       <c r="G47" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48">
@@ -3187,20 +3187,20 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>6.16</v>
+        <v>6.35</v>
       </c>
       <c r="E48" s="3" t="n">
         <v>5.69</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>7.54</v>
+        <v>7.78</v>
       </c>
       <c r="G48" t="n">
-        <v>336</v>
+        <v>317</v>
       </c>
     </row>
     <row r="49">
@@ -3216,20 +3216,20 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>7.43</v>
+        <v>7.51</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>7.09</v>
+        <v>7.2</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>7.96</v>
+        <v>7.99</v>
       </c>
       <c r="G49" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50">
@@ -3245,17 +3245,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>7.56</v>
+        <v>7.61</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>7.55</v>
+        <v>7.59</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>7.57</v>
+        <v>7.69</v>
       </c>
       <c r="G50" t="n">
         <v>15</v>
@@ -3274,20 +3274,20 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>6.29</v>
+        <v>6.42</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>5.57</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>6.99</v>
+        <v>7.19</v>
       </c>
       <c r="G51" t="n">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="52">
@@ -3303,20 +3303,20 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>6.35</v>
+        <v>6.65</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>5.39</v>
+        <v>5.59</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>8.970000000000001</v>
+        <v>8.99</v>
       </c>
       <c r="G52" t="n">
-        <v>1288</v>
+        <v>984</v>
       </c>
     </row>
     <row r="53">
@@ -3332,20 +3332,20 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>6.93</v>
+        <v>7.01</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>6.9</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>6.99</v>
+        <v>7.34</v>
       </c>
       <c r="G53" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54">
@@ -3361,20 +3361,20 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>6.94</v>
+        <v>7.05</v>
       </c>
       <c r="E54" s="3" t="n">
         <v>6.51</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>7.29</v>
+        <v>7.59</v>
       </c>
       <c r="G54" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55">
@@ -3390,20 +3390,20 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>124.47</v>
+        <v>7.43</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>114</v>
+        <v>6.99</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>135</v>
+        <v>8.26</v>
       </c>
       <c r="G55" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56">
@@ -3419,20 +3419,20 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>108.2</v>
+        <v>6.64</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>87.98999999999999</v>
+        <v>6.28</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>120</v>
+        <v>7.67</v>
       </c>
       <c r="G56" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57">
@@ -3448,20 +3448,20 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>129.1</v>
+        <v>6.35</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>115</v>
+        <v>6.24</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>139</v>
+        <v>6.85</v>
       </c>
       <c r="G57" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58">
@@ -3477,20 +3477,20 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>128.91</v>
+        <v>7.03</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>115</v>
+        <v>6.88</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>146</v>
+        <v>8.99</v>
       </c>
       <c r="G58" t="n">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59">
@@ -3506,20 +3506,20 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>116.38</v>
+        <v>6.7</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>93.98999999999999</v>
+        <v>6.13</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>150</v>
+        <v>9.92</v>
       </c>
       <c r="G59" t="n">
-        <v>164</v>
+        <v>224</v>
       </c>
     </row>
     <row r="60">
@@ -3535,20 +3535,20 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>112.6</v>
+        <v>6.94</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>98</v>
+        <v>5.84</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>135</v>
+        <v>7.38</v>
       </c>
       <c r="G60" t="n">
-        <v>80</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61">
@@ -3564,20 +3564,20 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>107.55</v>
+        <v>6.39</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>100</v>
+        <v>6.15</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>119.99</v>
+        <v>6.69</v>
       </c>
       <c r="G61" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62">
@@ -3593,20 +3593,20 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>105.21</v>
+        <v>6.39</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>95</v>
+        <v>6.03</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>130</v>
+        <v>7.23</v>
       </c>
       <c r="G62" t="n">
-        <v>63</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63">
@@ -3622,20 +3622,20 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>113.34</v>
+        <v>6.42</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>84</v>
+        <v>5.69</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>138</v>
+        <v>6.9</v>
       </c>
       <c r="G63" t="n">
-        <v>154</v>
+        <v>189</v>
       </c>
     </row>
     <row r="64">
@@ -3651,20 +3651,20 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>131.99</v>
+        <v>6.52</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>109.99</v>
+        <v>6.04</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>140</v>
+        <v>7.54</v>
       </c>
       <c r="G64" t="n">
-        <v>82</v>
+        <v>115</v>
       </c>
     </row>
     <row r="65">
@@ -3680,20 +3680,20 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>128.19</v>
+        <v>6.75</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>110</v>
+        <v>5.83</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>145</v>
+        <v>7.19</v>
       </c>
       <c r="G65" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="66">
@@ -3709,20 +3709,20 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>119.66</v>
+        <v>6.4</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>100</v>
+        <v>6.07</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>145</v>
+        <v>7.29</v>
       </c>
       <c r="G66" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="67">
@@ -3738,20 +3738,20 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>112.02</v>
+        <v>6.32</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>80</v>
+        <v>5.64</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>148</v>
+        <v>7.19</v>
       </c>
       <c r="G67" t="n">
-        <v>396</v>
+        <v>484</v>
       </c>
     </row>
     <row r="68">
@@ -3767,20 +3767,20 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>120.83</v>
+        <v>6.58</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>98.98999999999999</v>
+        <v>5.81</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>145</v>
+        <v>7.7</v>
       </c>
       <c r="G68" t="n">
-        <v>87</v>
+        <v>117</v>
       </c>
     </row>
     <row r="69">
@@ -3796,20 +3796,20 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>109.16</v>
+        <v>6.31</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>92.98999999999999</v>
+        <v>6.19</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>125</v>
+        <v>6.87</v>
       </c>
       <c r="G69" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70">
@@ -3825,20 +3825,20 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>114.25</v>
+        <v>6.57</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>94.98999999999999</v>
+        <v>5.59</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>135</v>
+        <v>7.38</v>
       </c>
       <c r="G70" t="n">
-        <v>250</v>
+        <v>291</v>
       </c>
     </row>
     <row r="71">
@@ -3854,20 +3854,20 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>104.88</v>
+        <v>6.88</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>86</v>
+        <v>6.13</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>130</v>
+        <v>7.99</v>
       </c>
       <c r="G71" t="n">
-        <v>130</v>
+        <v>192</v>
       </c>
     </row>
     <row r="72">
@@ -3883,20 +3883,20 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>112.09</v>
+        <v>6.71</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>100</v>
+        <v>6.19</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>137.99</v>
+        <v>6.99</v>
       </c>
       <c r="G72" t="n">
-        <v>40</v>
+        <v>59</v>
       </c>
     </row>
     <row r="73">
@@ -3912,20 +3912,20 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>104.72</v>
+        <v>6.59</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>84.98999999999999</v>
+        <v>6.08</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>151.99</v>
+        <v>7.39</v>
       </c>
       <c r="G73" t="n">
-        <v>209</v>
+        <v>322</v>
       </c>
     </row>
     <row r="74">
@@ -3941,20 +3941,20 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>115.71</v>
+        <v>6.76</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>95</v>
+        <v>6.22</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>130</v>
+        <v>7.59</v>
       </c>
       <c r="G74" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="75">
@@ -3970,20 +3970,20 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>118.59</v>
+        <v>6.16</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>94.98999999999999</v>
+        <v>5.69</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>161</v>
+        <v>7.54</v>
       </c>
       <c r="G75" t="n">
-        <v>276</v>
+        <v>336</v>
       </c>
     </row>
     <row r="76">
@@ -3999,20 +3999,20 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>127.94</v>
+        <v>7.43</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>112</v>
+        <v>7.09</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>148</v>
+        <v>7.96</v>
       </c>
       <c r="G76" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="77">
@@ -4028,20 +4028,20 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>140.8</v>
+        <v>7.56</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>130</v>
+        <v>7.55</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>156</v>
+        <v>7.57</v>
       </c>
       <c r="G77" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="78">
@@ -4057,20 +4057,20 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>122.23</v>
+        <v>6.29</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>94.98</v>
+        <v>5.57</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>145</v>
+        <v>6.99</v>
       </c>
       <c r="G78" t="n">
-        <v>94</v>
+        <v>159</v>
       </c>
     </row>
     <row r="79">
@@ -4086,20 +4086,20 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>116.84</v>
+        <v>6.35</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>79</v>
+        <v>5.39</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>150</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="G79" t="n">
-        <v>743</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="80">
@@ -4115,20 +4115,20 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>113.48</v>
+        <v>6.93</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>105</v>
+        <v>6.9</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>120</v>
+        <v>6.99</v>
       </c>
       <c r="G80" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="81">
@@ -4144,20 +4144,20 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>135.8</v>
+        <v>6.94</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>120</v>
+        <v>6.51</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>145</v>
+        <v>7.29</v>
       </c>
       <c r="G81" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
     </row>
     <row r="82">
@@ -4173,20 +4173,20 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>8.210000000000001</v>
+        <v>124.47</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>7.89</v>
+        <v>114</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>8.85</v>
+        <v>135</v>
       </c>
       <c r="G82" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="83">
@@ -4202,20 +4202,20 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>7.33</v>
+        <v>108.2</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>7.18</v>
+        <v>87.98999999999999</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>8.4</v>
+        <v>120</v>
       </c>
       <c r="G83" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="84">
@@ -4231,20 +4231,20 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>7.21</v>
+        <v>129.1</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>7.12</v>
+        <v>115</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>7.9</v>
+        <v>139</v>
       </c>
       <c r="G84" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="85">
@@ -4260,20 +4260,20 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>7.22</v>
+        <v>128.91</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>6.98</v>
+        <v>115</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>8.99</v>
+        <v>146</v>
       </c>
       <c r="G85" t="n">
-        <v>37</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86">
@@ -4289,20 +4289,20 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>7.51</v>
+        <v>116.38</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>6.79</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>8.99</v>
+        <v>150</v>
       </c>
       <c r="G86" t="n">
-        <v>175</v>
+        <v>164</v>
       </c>
     </row>
     <row r="87">
@@ -4318,20 +4318,20 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>7.3</v>
+        <v>112.6</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>6.15</v>
+        <v>98</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>8.4</v>
+        <v>135</v>
       </c>
       <c r="G87" t="n">
-        <v>129</v>
+        <v>80</v>
       </c>
     </row>
     <row r="88">
@@ -4347,20 +4347,20 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>7.44</v>
+        <v>107.55</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>7.05</v>
+        <v>100</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>7.69</v>
+        <v>119.99</v>
       </c>
       <c r="G88" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="89">
@@ -4376,20 +4376,20 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>6.87</v>
+        <v>105.21</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>6.19</v>
+        <v>95</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>7.29</v>
+        <v>130</v>
       </c>
       <c r="G89" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="90">
@@ -4405,20 +4405,20 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>7.3</v>
+        <v>113.34</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>6.62</v>
+        <v>84</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>7.99</v>
+        <v>138</v>
       </c>
       <c r="G90" t="n">
-        <v>141</v>
+        <v>154</v>
       </c>
     </row>
     <row r="91">
@@ -4434,20 +4434,20 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>7.47</v>
+        <v>131.99</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>6.87</v>
+        <v>109.99</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>8.390000000000001</v>
+        <v>140</v>
       </c>
       <c r="G91" t="n">
-        <v>98</v>
+        <v>82</v>
       </c>
     </row>
     <row r="92">
@@ -4463,20 +4463,20 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>7.6</v>
+        <v>128.19</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>6.89</v>
+        <v>110</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>8.949999999999999</v>
+        <v>145</v>
       </c>
       <c r="G92" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
     </row>
     <row r="93">
@@ -4492,20 +4492,20 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>7.34</v>
+        <v>119.66</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>7.09</v>
+        <v>100</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>7.93</v>
+        <v>145</v>
       </c>
       <c r="G93" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
     </row>
     <row r="94">
@@ -4521,20 +4521,20 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>7.05</v>
+        <v>112.02</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>6.39</v>
+        <v>80</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>8.289999999999999</v>
+        <v>148</v>
       </c>
       <c r="G94" t="n">
-        <v>334</v>
+        <v>396</v>
       </c>
     </row>
     <row r="95">
@@ -4550,20 +4550,20 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>7.53</v>
+        <v>120.83</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>6.65</v>
+        <v>98.98999999999999</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>145</v>
       </c>
       <c r="G95" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="96">
@@ -4579,20 +4579,20 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>7.28</v>
+        <v>109.16</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>6.95</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>7.8</v>
+        <v>125</v>
       </c>
       <c r="G96" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="97">
@@ -4608,20 +4608,20 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>7.36</v>
+        <v>114.25</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>6.79</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>8.49</v>
+        <v>135</v>
       </c>
       <c r="G97" t="n">
-        <v>203</v>
+        <v>250</v>
       </c>
     </row>
     <row r="98">
@@ -4637,20 +4637,20 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>7.27</v>
+        <v>104.88</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>6.69</v>
+        <v>86</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>8.34</v>
+        <v>130</v>
       </c>
       <c r="G98" t="n">
-        <v>165</v>
+        <v>130</v>
       </c>
     </row>
     <row r="99">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>7.7</v>
+        <v>112.09</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>7.49</v>
+        <v>100</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>8.25</v>
+        <v>137.99</v>
       </c>
       <c r="G99" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="100">
@@ -4695,20 +4695,20 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>7.15</v>
+        <v>104.72</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>5.89</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>8.19</v>
+        <v>151.99</v>
       </c>
       <c r="G100" t="n">
-        <v>225</v>
+        <v>209</v>
       </c>
     </row>
     <row r="101">
@@ -4724,20 +4724,20 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>7.5</v>
+        <v>115.71</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>6.99</v>
+        <v>95</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>8.289999999999999</v>
+        <v>130</v>
       </c>
       <c r="G101" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="102">
@@ -4753,20 +4753,20 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>7.16</v>
+        <v>118.59</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>6.45</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>8.289999999999999</v>
+        <v>161</v>
       </c>
       <c r="G102" t="n">
-        <v>235</v>
+        <v>276</v>
       </c>
     </row>
     <row r="103">
@@ -4782,20 +4782,20 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>7.57</v>
+        <v>127.94</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>6.99</v>
+        <v>112</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>7.99</v>
+        <v>148</v>
       </c>
       <c r="G103" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="104">
@@ -4811,20 +4811,20 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>7.6</v>
+        <v>140.8</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>7.25</v>
+        <v>130</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>7.65</v>
+        <v>156</v>
       </c>
       <c r="G104" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="105">
@@ -4840,20 +4840,20 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>7.23</v>
+        <v>122.23</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>6.69</v>
+        <v>94.98</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>7.99</v>
+        <v>145</v>
       </c>
       <c r="G105" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="106">
@@ -4869,20 +4869,20 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>7.32</v>
+        <v>116.84</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>6.29</v>
+        <v>79</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>9.99</v>
+        <v>150</v>
       </c>
       <c r="G106" t="n">
-        <v>864</v>
+        <v>743</v>
       </c>
     </row>
     <row r="107">
@@ -4898,20 +4898,20 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="D107" s="3" t="n">
-        <v>7.33</v>
+        <v>113.48</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>7.29</v>
+        <v>105</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>7.59</v>
+        <v>120</v>
       </c>
       <c r="G107" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
     </row>
     <row r="108">
@@ -4927,19 +4927,2020 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
+          <t>GLP</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="n">
+        <v>135.8</v>
+      </c>
+      <c r="E108" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>145</v>
+      </c>
+      <c r="G108" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="G109" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="E110" s="3" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="G110" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="E111" s="3" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="G111" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="E112" s="3" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="G112" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="E113" s="3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="G113" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="E114" s="3" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F114" s="3" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="G114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="E115" s="3" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="F115" s="3" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="G115" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="E116" s="3" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="F116" s="3" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="G116" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="E117" s="3" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="F117" s="3" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="G117" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="E118" s="3" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="F118" s="3" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="G118" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="E119" s="3" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="F119" s="3" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="G119" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="E120" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F120" s="3" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="G120" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="E121" s="3" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="F121" s="3" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="G121" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E122" s="3" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="F122" s="3" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="G122" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="E123" s="3" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F123" s="3" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="G123" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>GNV</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="E124" s="3" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="F124" s="3" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="G124" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="E125" s="3" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="F125" s="3" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G125" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="E126" s="3" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="F126" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G126" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="E127" s="3" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F127" s="3" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="G127" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="E128" s="3" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="F128" s="3" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="G128" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E129" s="3" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="F129" s="3" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="G129" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="E130" s="3" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="F130" s="3" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="G130" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="E131" s="3" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="F131" s="3" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="G131" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="E132" s="3" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="F132" s="3" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="G132" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="E133" s="3" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F133" s="3" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="G133" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="E134" s="3" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="F134" s="3" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="G134" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E135" s="3" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="F135" s="3" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="G135" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="E136" s="3" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="F136" s="3" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="G136" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="E137" s="3" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="F137" s="3" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G137" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="E138" s="3" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F138" s="3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G138" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="E139" s="3" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F139" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G139" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="E140" s="3" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="F140" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G140" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="E141" s="3" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="F141" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G141" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="E142" s="3" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="F142" s="3" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="G142" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="E143" s="3" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="F143" s="3" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="G143" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="E144" s="3" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="F144" s="3" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="G144" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="E145" s="3" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="F145" s="3" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="G145" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="F146" s="3" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="G146" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="E147" s="3" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F147" s="3" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="G147" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="E148" s="3" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F148" s="3" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="G148" t="n">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="E149" s="3" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F149" s="3" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="G149" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="F150" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G150" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
           <t>OLEO DIESEL S10</t>
         </is>
       </c>
-      <c r="D108" s="3" t="n">
+      <c r="D151" s="3" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="E151" s="3" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="F151" s="3" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="G151" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="F152" s="3" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G152" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="E153" s="3" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F153" s="3" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G153" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="E154" s="3" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="F154" s="3" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="G154" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E155" s="3" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="F155" s="3" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="G155" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E156" s="3" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="F156" s="3" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G156" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="E157" s="3" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="F157" s="3" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="G157" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="E158" s="3" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="F158" s="3" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="G158" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E159" s="3" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="F159" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G159" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="E160" s="3" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="F160" s="3" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="G160" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E161" s="3" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="F161" s="3" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="G161" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>CENTRO OESTE</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="E162" s="3" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="F162" s="3" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="G162" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="E163" s="3" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="F163" s="3" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="G163" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="E164" s="3" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F164" s="3" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G164" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="E165" s="3" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="F165" s="3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G165" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="E166" s="3" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="F166" s="3" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="G166" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="E167" s="3" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="F167" s="3" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="G167" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E168" s="3" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="F168" s="3" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="G168" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="E169" s="3" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="F169" s="3" t="n">
+        <v>8.19</v>
+      </c>
+      <c r="G169" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E170" s="3" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F170" s="3" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="G170" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="E171" s="3" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="F171" s="3" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="G171" t="n">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="E172" s="3" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F172" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G172" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E173" s="3" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F173" s="3" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="G173" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>SUL</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="E174" s="3" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="F174" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G174" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>SUDESTE</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="E175" s="3" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="F175" s="3" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="G175" t="n">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>NORDESTE</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="E176" s="3" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="F176" s="3" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="G176" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>OLEO DIESEL S10</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="n">
         <v>7.42</v>
       </c>
-      <c r="E108" s="3" t="n">
+      <c r="E177" s="3" t="n">
         <v>6.96</v>
       </c>
-      <c r="F108" s="3" t="n">
+      <c r="F177" s="3" t="n">
         <v>7.99</v>
       </c>
-      <c r="G108" t="n">
+      <c r="G177" t="n">
         <v>41</v>
       </c>
     </row>

</xml_diff>